<commit_message>
Add Disco description column to spreadsheet template and manual
Add a desc (概要) column to the Disco sheet, positioned between
tracks and 公開, so the album detail page's overview text (shown
between release info and the tracklist) can be edited from Google
Sheets. Update 更新マニュアル.md with input instructions for the
new column and a note that clients only need to touch the Google
Sheet, not GitHub/Vercel/Apps Script.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/howling-way-スプレッドシートひな型.xlsx
+++ b/howling-way-スプレッドシートひな型.xlsx
@@ -1195,20 +1195,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>【作品】CD・配信作品の情報を入力すると、サイトのDiscographyに表示されます。上から順（新しい順がおすすめ）に表示されます。</t>
+          <t>【作品】CD・配信作品の情報を入力すると、サイトのDiscographyに表示されます。上から順（新しい順がおすすめ）に表示されます。「概要」を入力すると、作品詳細ページのリリース情報とTRACKLISTの間に誌明文が表示されます（空樓でも可）。</t>
         </is>
       </c>
     </row>
@@ -1235,6 +1236,11 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>desc</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>公開</t>
         </is>
       </c>
@@ -1262,6 +1268,11 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
+          <t>概要</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
           <t>公開</t>
         </is>
       </c>
@@ -1289,6 +1300,11 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
+          <t>Howling way 2作目となるミニアルバム。過去最多の全7曲を収録し、バンドの新たな一面を切り押いた作品。</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
           <t>TRUE</t>
         </is>
       </c>
@@ -1314,7 +1330,7 @@
           <t>beautiful</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -1341,7 +1357,7 @@
           <t>ラストラリー / HEART</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -1368,7 +1384,7 @@
           <t>ギフト / 人の子のため / いつかすべてを / スーツ / スーパーヒーロー / 遠吠え / 未完成ライダー</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -1376,10 +1392,10 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E4:E200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F4:F200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>